<commit_message>
data: se anonimizan los .xlsx de muestra de Momento 4 y Participación
Estos archivos ya no los lee la app —los datos viven en Postgres— pero
seguían en el repo con nombres, apellidos, cédula y código de estudiante
reales. Se vacían esos valores dejando encabezados, posiciones y el resto
de columnas intactos, así que siguen sirviendo como muestra del formato de
entrada.
</commit_message>
<xml_diff>
--- a/data/source-participacon-momoento4-planeacion-teritorial/participacion2026-18-08.xlsx
+++ b/data/source-participacon-momoento4-planeacion-teritorial/participacion2026-18-08.xlsx
@@ -121,10 +121,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
+        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
+        <a:font script="Hans" typeface="å®ä½"/>
+        <a:font script="Hant" typeface="æ°ç´°æé«"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -156,10 +156,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
+        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
+        <a:font script="Hans" typeface="å®ä½"/>
+        <a:font script="Hant" typeface="æ°ç´°æé«"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -481,7 +481,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C2" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -511,13 +511,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L2" t="str">
-        <v>PACHECO MEDINA LUZ GINNETH</v>
+        <v/>
       </c>
       <c r="M2" t="str">
-        <v>LUZ GINNETH</v>
+        <v/>
       </c>
       <c r="N2" t="str">
-        <v>PACHECO MEDINA</v>
+        <v/>
       </c>
       <c r="O2">
         <v>50</v>
@@ -546,7 +546,7 @@
         <v>0</v>
       </c>
       <c r="B3" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C3" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -576,13 +576,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L3" t="str">
-        <v>MANRIQUE LARA ERIN HAROLD ERNESTO</v>
+        <v/>
       </c>
       <c r="M3" t="str">
-        <v>ERIN HAROLD ERNESTO</v>
+        <v/>
       </c>
       <c r="N3" t="str">
-        <v>MANRIQUE LARA</v>
+        <v/>
       </c>
       <c r="O3">
         <v>40</v>
@@ -611,7 +611,7 @@
         <v>0</v>
       </c>
       <c r="B4" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C4" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -641,13 +641,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L4" t="str">
-        <v>PEÑUELA CABALLERO VIVIANA ANDREA</v>
+        <v/>
       </c>
       <c r="M4" t="str">
-        <v>VIVIANA ANDREA</v>
+        <v/>
       </c>
       <c r="N4" t="str">
-        <v>PEÑUELA CABALLERO</v>
+        <v/>
       </c>
       <c r="O4">
         <v>38</v>
@@ -676,7 +676,7 @@
         <v>0</v>
       </c>
       <c r="B5" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C5" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -706,13 +706,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L5" t="str">
-        <v>PARAMO ARAGON JENNY ALEZANDRA</v>
+        <v/>
       </c>
       <c r="M5" t="str">
-        <v>JENNY ALEZANDRA</v>
+        <v/>
       </c>
       <c r="N5" t="str">
-        <v>PARAMO ARAGON</v>
+        <v/>
       </c>
       <c r="O5">
         <v>48</v>
@@ -732,7 +732,7 @@
         <v>0</v>
       </c>
       <c r="B6" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C6" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -762,13 +762,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L6" t="str">
-        <v>TOVAR BARACALDO YODY YEDILMA</v>
+        <v/>
       </c>
       <c r="M6" t="str">
-        <v>YODY YEDILMA</v>
+        <v/>
       </c>
       <c r="N6" t="str">
-        <v>TOVAR BARACALDO</v>
+        <v/>
       </c>
       <c r="O6">
         <v>37</v>
@@ -788,7 +788,7 @@
         <v>0</v>
       </c>
       <c r="B7" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C7" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -818,13 +818,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L7" t="str">
-        <v>VERGARA BELTRAN SAMIR FERNANDO</v>
+        <v/>
       </c>
       <c r="M7" t="str">
-        <v>SAMIR FERNANDO</v>
+        <v/>
       </c>
       <c r="N7" t="str">
-        <v>VERGARA BELTRAN</v>
+        <v/>
       </c>
       <c r="O7">
         <v>53</v>
@@ -853,7 +853,7 @@
         <v>0</v>
       </c>
       <c r="B8" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C8" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -883,13 +883,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L8" t="str">
-        <v>PEÑA CAÑÓN EHIDY ROCIO</v>
+        <v/>
       </c>
       <c r="M8" t="str">
-        <v>EHIDY ROCIO</v>
+        <v/>
       </c>
       <c r="N8" t="str">
-        <v>PEÑA CAÑÓN</v>
+        <v/>
       </c>
       <c r="O8">
         <v>39</v>
@@ -918,7 +918,7 @@
         <v>0</v>
       </c>
       <c r="B9" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C9" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -948,13 +948,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L9" t="str">
-        <v>CASTAÑEDA CELEITA WILLIAM ANDRES</v>
+        <v/>
       </c>
       <c r="M9" t="str">
-        <v>WILLIAM ANDRES</v>
+        <v/>
       </c>
       <c r="N9" t="str">
-        <v>CASTAÑEDA CELEITA</v>
+        <v/>
       </c>
       <c r="O9">
         <v>44</v>
@@ -974,7 +974,7 @@
         <v>0</v>
       </c>
       <c r="B10" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C10" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -1004,13 +1004,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L10" t="str">
-        <v>BAUTISTA GAONA JUAN ESTEBAN</v>
+        <v/>
       </c>
       <c r="M10" t="str">
-        <v>JUAN ESTEBAN</v>
+        <v/>
       </c>
       <c r="N10" t="str">
-        <v>BAUTISTA GAONA</v>
+        <v/>
       </c>
       <c r="O10">
         <v>29</v>
@@ -1024,7 +1024,7 @@
         <v>0</v>
       </c>
       <c r="B11" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C11" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -1054,13 +1054,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L11" t="str">
-        <v>TARAZONA APONTE DENNISE ALEJANDRA</v>
+        <v/>
       </c>
       <c r="M11" t="str">
-        <v>DENNISE ALEJANDRA</v>
+        <v/>
       </c>
       <c r="N11" t="str">
-        <v>TARAZONA APONTE</v>
+        <v/>
       </c>
       <c r="O11">
         <v>32</v>
@@ -1089,7 +1089,7 @@
         <v>0</v>
       </c>
       <c r="B12" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C12" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -1119,13 +1119,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L12" t="str">
-        <v>GUZMAN SALGUERO ADELINA</v>
+        <v/>
       </c>
       <c r="M12" t="str">
-        <v>ADELINA</v>
+        <v/>
       </c>
       <c r="N12" t="str">
-        <v>GUZMAN SALGUERO</v>
+        <v/>
       </c>
       <c r="O12">
         <v>59</v>
@@ -1154,7 +1154,7 @@
         <v>0</v>
       </c>
       <c r="B13" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C13" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -1184,13 +1184,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L13" t="str">
-        <v>SASTOQUE RINCON FABIO ALEJANDRO</v>
+        <v/>
       </c>
       <c r="M13" t="str">
-        <v>FABIO ALEJANDRO</v>
+        <v/>
       </c>
       <c r="N13" t="str">
-        <v>SASTOQUE RINCON</v>
+        <v/>
       </c>
       <c r="O13">
         <v>27</v>
@@ -1219,7 +1219,7 @@
         <v>0</v>
       </c>
       <c r="B14" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C14" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -1249,13 +1249,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L14" t="str">
-        <v>AGUDELO RODRIGUEZ NOHORA LILIANA</v>
+        <v/>
       </c>
       <c r="M14" t="str">
-        <v>NOHORA LILIANA</v>
+        <v/>
       </c>
       <c r="N14" t="str">
-        <v>AGUDELO RODRIGUEZ</v>
+        <v/>
       </c>
       <c r="O14">
         <v>38</v>
@@ -1275,7 +1275,7 @@
         <v>0</v>
       </c>
       <c r="B15" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C15" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -1305,13 +1305,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L15" t="str">
-        <v>GRACIA GIL JAVIER HERNANDO</v>
+        <v/>
       </c>
       <c r="M15" t="str">
-        <v>JAVIER HERNANDO</v>
+        <v/>
       </c>
       <c r="N15" t="str">
-        <v>GRACIA GIL</v>
+        <v/>
       </c>
       <c r="O15">
         <v>51</v>
@@ -1331,7 +1331,7 @@
         <v>0</v>
       </c>
       <c r="B16" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C16" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -1361,13 +1361,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L16" t="str">
-        <v>GARZON SOCHE MARIA NANCY</v>
+        <v/>
       </c>
       <c r="M16" t="str">
-        <v>MARIA NANCY</v>
+        <v/>
       </c>
       <c r="N16" t="str">
-        <v>GARZON SOCHE</v>
+        <v/>
       </c>
       <c r="O16">
         <v>60</v>
@@ -1387,7 +1387,7 @@
         <v>0</v>
       </c>
       <c r="B17" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C17" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -1417,13 +1417,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L17" t="str">
-        <v>BELLO MOJICA ELIANA CONSTANZA</v>
+        <v/>
       </c>
       <c r="M17" t="str">
-        <v>ELIANA CONSTANZA</v>
+        <v/>
       </c>
       <c r="N17" t="str">
-        <v>BELLO MOJICA</v>
+        <v/>
       </c>
       <c r="O17">
         <v>38</v>
@@ -1452,7 +1452,7 @@
         <v>0</v>
       </c>
       <c r="B18" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C18" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -1482,13 +1482,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L18" t="str">
-        <v>MORENO RODRIGUEZ FABIAN</v>
+        <v/>
       </c>
       <c r="M18" t="str">
-        <v>FABIAN</v>
+        <v/>
       </c>
       <c r="N18" t="str">
-        <v>MORENO RODRIGUEZ</v>
+        <v/>
       </c>
       <c r="O18">
         <v>45</v>
@@ -1517,7 +1517,7 @@
         <v>0</v>
       </c>
       <c r="B19" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C19" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -1547,13 +1547,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L19" t="str">
-        <v>MORENO SANDOVAL JOHN ALEXANDER</v>
+        <v/>
       </c>
       <c r="M19" t="str">
-        <v>JOHN ALEXANDER</v>
+        <v/>
       </c>
       <c r="N19" t="str">
-        <v>MORENO SANDOVAL</v>
+        <v/>
       </c>
       <c r="O19">
         <v>46</v>
@@ -1573,7 +1573,7 @@
         <v>0</v>
       </c>
       <c r="B20" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C20" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -1603,13 +1603,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L20" t="str">
-        <v>VELASQUEZ RAMIREZ GUSTAVO</v>
+        <v/>
       </c>
       <c r="M20" t="str">
-        <v>GUSTAVO</v>
+        <v/>
       </c>
       <c r="N20" t="str">
-        <v>VELASQUEZ RAMIREZ</v>
+        <v/>
       </c>
       <c r="O20">
         <v>56</v>
@@ -1638,7 +1638,7 @@
         <v>0</v>
       </c>
       <c r="B21" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C21" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -1668,13 +1668,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L21" t="str">
-        <v>PAVA VARGAS ANDRES FERNANDO</v>
+        <v/>
       </c>
       <c r="M21" t="str">
-        <v>ANDRES FERNANDO</v>
+        <v/>
       </c>
       <c r="N21" t="str">
-        <v>PAVA VARGAS</v>
+        <v/>
       </c>
       <c r="O21">
         <v>32</v>
@@ -1703,7 +1703,7 @@
         <v>0</v>
       </c>
       <c r="B22" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C22" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -1733,13 +1733,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L22" t="str">
-        <v>RUBIO BUITRAGO NATHALIA CAROLINA</v>
+        <v/>
       </c>
       <c r="M22" t="str">
-        <v>NATHALIA CAROLINA</v>
+        <v/>
       </c>
       <c r="N22" t="str">
-        <v>RUBIO BUITRAGO</v>
+        <v/>
       </c>
       <c r="O22">
         <v>39</v>
@@ -1768,7 +1768,7 @@
         <v>0</v>
       </c>
       <c r="B23" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C23" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -1798,13 +1798,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L23" t="str">
-        <v>RINCÓN FORERO ADRIANA MARCELA</v>
+        <v/>
       </c>
       <c r="M23" t="str">
-        <v>ADRIANA MARCELA</v>
+        <v/>
       </c>
       <c r="N23" t="str">
-        <v>RINCÓN FORERO</v>
+        <v/>
       </c>
       <c r="O23">
         <v>36</v>
@@ -1833,7 +1833,7 @@
         <v>0</v>
       </c>
       <c r="B24" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C24" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -1863,13 +1863,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L24" t="str">
-        <v>ORTEGA ORTEGA RAFAEL</v>
+        <v/>
       </c>
       <c r="M24" t="str">
-        <v>RAFAEL</v>
+        <v/>
       </c>
       <c r="N24" t="str">
-        <v>ORTEGA ORTEGA</v>
+        <v/>
       </c>
       <c r="O24">
         <v>38</v>
@@ -1898,7 +1898,7 @@
         <v>0</v>
       </c>
       <c r="B25" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C25" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -1928,13 +1928,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L25" t="str">
-        <v>CASAS MÉNDEZ YENY LILIANA</v>
+        <v/>
       </c>
       <c r="M25" t="str">
-        <v>YENY LILIANA</v>
+        <v/>
       </c>
       <c r="N25" t="str">
-        <v>CASAS MÉNDEZ</v>
+        <v/>
       </c>
       <c r="O25">
         <v>41</v>
@@ -1963,7 +1963,7 @@
         <v>0</v>
       </c>
       <c r="B26" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C26" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -1993,13 +1993,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L26" t="str">
-        <v>YAYA CHACON ZULMA CISNEY</v>
+        <v/>
       </c>
       <c r="M26" t="str">
-        <v>ZULMA CISNEY</v>
+        <v/>
       </c>
       <c r="N26" t="str">
-        <v>YAYA CHACON</v>
+        <v/>
       </c>
       <c r="O26">
         <v>46</v>
@@ -2028,7 +2028,7 @@
         <v>0</v>
       </c>
       <c r="B27" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C27" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -2058,13 +2058,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L27" t="str">
-        <v>GARCÍA BALLÉN GLORIA ISABEL</v>
+        <v/>
       </c>
       <c r="M27" t="str">
-        <v>GLORIA ISABEL</v>
+        <v/>
       </c>
       <c r="N27" t="str">
-        <v>GARCÍA BALLÉN</v>
+        <v/>
       </c>
       <c r="O27">
         <v>44</v>
@@ -2084,7 +2084,7 @@
         <v>0</v>
       </c>
       <c r="B28" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C28" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -2114,13 +2114,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L28" t="str">
-        <v>MUNEVAR MORENO RODOLFO ANTONIO</v>
+        <v/>
       </c>
       <c r="M28" t="str">
-        <v>RODOLFO ANTONIO</v>
+        <v/>
       </c>
       <c r="N28" t="str">
-        <v>MUNEVAR MORENO</v>
+        <v/>
       </c>
       <c r="O28">
         <v>48</v>
@@ -2149,7 +2149,7 @@
         <v>0</v>
       </c>
       <c r="B29" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C29" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -2179,13 +2179,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L29" t="str">
-        <v>CASTRO FAJARDO HERMES</v>
+        <v/>
       </c>
       <c r="M29" t="str">
-        <v>HERMES</v>
+        <v/>
       </c>
       <c r="N29" t="str">
-        <v>CASTRO FAJARDO</v>
+        <v/>
       </c>
       <c r="O29">
         <v>48</v>
@@ -2214,7 +2214,7 @@
         <v>0</v>
       </c>
       <c r="B30" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C30" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -2244,13 +2244,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L30" t="str">
-        <v>ROA GUERRERO EDGAR EDUARDO</v>
+        <v/>
       </c>
       <c r="M30" t="str">
-        <v>EDGAR EDUARDO</v>
+        <v/>
       </c>
       <c r="N30" t="str">
-        <v>ROA GUERRERO</v>
+        <v/>
       </c>
       <c r="O30">
         <v>41</v>
@@ -2270,7 +2270,7 @@
         <v>0</v>
       </c>
       <c r="B31" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C31" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -2300,13 +2300,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L31" t="str">
-        <v>CAICEDO BELLO EDWIN ROMAN</v>
+        <v/>
       </c>
       <c r="M31" t="str">
-        <v>EDWIN ROMAN</v>
+        <v/>
       </c>
       <c r="N31" t="str">
-        <v>CAICEDO BELLO</v>
+        <v/>
       </c>
       <c r="O31">
         <v>37</v>
@@ -2335,7 +2335,7 @@
         <v>0</v>
       </c>
       <c r="B32" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C32" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -2365,13 +2365,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L32" t="str">
-        <v>PABON QUINTERO JESUS ENRIQUE</v>
+        <v/>
       </c>
       <c r="M32" t="str">
-        <v>JESUS ENRIQUE</v>
+        <v/>
       </c>
       <c r="N32" t="str">
-        <v>PABON QUINTERO</v>
+        <v/>
       </c>
       <c r="O32">
         <v>45</v>
@@ -2391,7 +2391,7 @@
         <v>0</v>
       </c>
       <c r="B33" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C33" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -2421,13 +2421,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L33" t="str">
-        <v>LANCHEROS CAÑON WILSON ARMANDO</v>
+        <v/>
       </c>
       <c r="M33" t="str">
-        <v>WILSON ARMANDO</v>
+        <v/>
       </c>
       <c r="N33" t="str">
-        <v>LANCHEROS CAÑON</v>
+        <v/>
       </c>
       <c r="O33">
         <v>55</v>
@@ -2456,7 +2456,7 @@
         <v>0</v>
       </c>
       <c r="B34" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C34" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -2486,13 +2486,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L34" t="str">
-        <v>SIMIJACA SALCEDO DIEGO FERNANDO</v>
+        <v/>
       </c>
       <c r="M34" t="str">
-        <v>DIEGO FERNANDO</v>
+        <v/>
       </c>
       <c r="N34" t="str">
-        <v>SIMIJACA SALCEDO</v>
+        <v/>
       </c>
       <c r="O34">
         <v>39</v>
@@ -2521,7 +2521,7 @@
         <v>0</v>
       </c>
       <c r="B35" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C35" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -2551,13 +2551,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L35" t="str">
-        <v>NIÑO MENDEZ OSCAR ADOLFO</v>
+        <v/>
       </c>
       <c r="M35" t="str">
-        <v>OSCAR ADOLFO</v>
+        <v/>
       </c>
       <c r="N35" t="str">
-        <v>NIÑO MENDEZ</v>
+        <v/>
       </c>
       <c r="O35">
         <v>47</v>
@@ -2577,7 +2577,7 @@
         <v>0</v>
       </c>
       <c r="B36" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C36" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -2607,13 +2607,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L36" t="str">
-        <v>RODRÍGUEZ MONTES JUAN CAMILO</v>
+        <v/>
       </c>
       <c r="M36" t="str">
-        <v>JUAN CAMILO</v>
+        <v/>
       </c>
       <c r="N36" t="str">
-        <v>RODRÍGUEZ MONTES</v>
+        <v/>
       </c>
       <c r="O36">
         <v>29</v>
@@ -2642,7 +2642,7 @@
         <v>0</v>
       </c>
       <c r="B37" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C37" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -2672,13 +2672,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L37" t="str">
-        <v>SANCHEZ SARRAZOLA LUIS EDUARDO</v>
+        <v/>
       </c>
       <c r="M37" t="str">
-        <v>LUIS EDUARDO</v>
+        <v/>
       </c>
       <c r="N37" t="str">
-        <v>SANCHEZ SARRAZOLA</v>
+        <v/>
       </c>
       <c r="O37">
         <v>71</v>
@@ -2707,7 +2707,7 @@
         <v>0</v>
       </c>
       <c r="B38" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C38" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -2737,13 +2737,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L38" t="str">
-        <v>VELÁSQUEZ PARRA IVÁN OLIMPO</v>
+        <v/>
       </c>
       <c r="M38" t="str">
-        <v>IVÁN OLIMPO</v>
+        <v/>
       </c>
       <c r="N38" t="str">
-        <v>VELÁSQUEZ PARRA</v>
+        <v/>
       </c>
       <c r="O38">
         <v>58</v>
@@ -2772,7 +2772,7 @@
         <v>0</v>
       </c>
       <c r="B39" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C39" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -2802,13 +2802,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L39" t="str">
-        <v>FRANCO GONZALEZ NESTOR JOSUE</v>
+        <v/>
       </c>
       <c r="M39" t="str">
-        <v>NESTOR JOSUE</v>
+        <v/>
       </c>
       <c r="N39" t="str">
-        <v>FRANCO GONZALEZ</v>
+        <v/>
       </c>
       <c r="O39">
         <v>49</v>
@@ -2837,7 +2837,7 @@
         <v>0</v>
       </c>
       <c r="B40" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C40" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -2867,13 +2867,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L40" t="str">
-        <v>BAYONA ALBARRACÍN JOHANA ALEXANDRA</v>
+        <v/>
       </c>
       <c r="M40" t="str">
-        <v>JOHANA ALEXANDRA</v>
+        <v/>
       </c>
       <c r="N40" t="str">
-        <v>BAYONA ALBARRACÍN</v>
+        <v/>
       </c>
       <c r="O40">
         <v>43</v>
@@ -2902,7 +2902,7 @@
         <v>0</v>
       </c>
       <c r="B41" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C41" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -2932,13 +2932,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L41" t="str">
-        <v>CASTIBLANCO FORERO LEDIS JOHANA</v>
+        <v/>
       </c>
       <c r="M41" t="str">
-        <v>LEDIS JOHANA</v>
+        <v/>
       </c>
       <c r="N41" t="str">
-        <v>CASTIBLANCO FORERO</v>
+        <v/>
       </c>
       <c r="O41">
         <v>40</v>
@@ -2967,7 +2967,7 @@
         <v>0</v>
       </c>
       <c r="B42" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C42" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -2997,13 +2997,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L42" t="str">
-        <v>PÉREZ GAVIRIA YULIANA</v>
+        <v/>
       </c>
       <c r="M42" t="str">
-        <v>YULIANA</v>
+        <v/>
       </c>
       <c r="N42" t="str">
-        <v>PÉREZ GAVIRIA</v>
+        <v/>
       </c>
       <c r="O42">
         <v>41</v>
@@ -3032,7 +3032,7 @@
         <v>0</v>
       </c>
       <c r="B43" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C43" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -3062,13 +3062,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L43" t="str">
-        <v>USAQUEN RIVERA JENNIFER LORENA</v>
+        <v/>
       </c>
       <c r="M43" t="str">
-        <v>JENNIFER LORENA</v>
+        <v/>
       </c>
       <c r="N43" t="str">
-        <v>USAQUEN RIVERA</v>
+        <v/>
       </c>
       <c r="O43">
         <v>31</v>
@@ -3097,7 +3097,7 @@
         <v>0</v>
       </c>
       <c r="B44" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C44" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -3127,13 +3127,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L44" t="str">
-        <v>LARA RODRIGUEZ LUISA JOHANNA</v>
+        <v/>
       </c>
       <c r="M44" t="str">
-        <v>LUISA JOHANNA</v>
+        <v/>
       </c>
       <c r="N44" t="str">
-        <v>LARA RODRIGUEZ</v>
+        <v/>
       </c>
       <c r="O44">
         <v>44</v>
@@ -3162,7 +3162,7 @@
         <v>0</v>
       </c>
       <c r="B45" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C45" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -3192,13 +3192,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L45" t="str">
-        <v>ALONSO GOMEZ DORA CONSTANZA</v>
+        <v/>
       </c>
       <c r="M45" t="str">
-        <v>DORA CONSTANZA</v>
+        <v/>
       </c>
       <c r="N45" t="str">
-        <v>ALONSO GOMEZ</v>
+        <v/>
       </c>
       <c r="O45">
         <v>47</v>
@@ -3227,7 +3227,7 @@
         <v>0</v>
       </c>
       <c r="B46" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C46" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -3257,13 +3257,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L46" t="str">
-        <v>MURCIA CASTRO STEFANIA</v>
+        <v/>
       </c>
       <c r="M46" t="str">
-        <v>STEFANIA</v>
+        <v/>
       </c>
       <c r="N46" t="str">
-        <v>MURCIA CASTRO</v>
+        <v/>
       </c>
       <c r="O46">
         <v>28</v>
@@ -3292,7 +3292,7 @@
         <v>0</v>
       </c>
       <c r="B47" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C47" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -3322,13 +3322,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L47" t="str">
-        <v>MONROY GONZÁLEZ MARBEL YULIETH</v>
+        <v/>
       </c>
       <c r="M47" t="str">
-        <v>MARBEL YULIETH</v>
+        <v/>
       </c>
       <c r="N47" t="str">
-        <v>MONROY GONZÁLEZ</v>
+        <v/>
       </c>
       <c r="O47">
         <v>38</v>
@@ -3357,7 +3357,7 @@
         <v>0</v>
       </c>
       <c r="B48" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C48" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -3387,13 +3387,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L48" t="str">
-        <v>TORRES ESPITIA ADRIANA ASENCION</v>
+        <v/>
       </c>
       <c r="M48" t="str">
-        <v>ADRIANA ASENCION</v>
+        <v/>
       </c>
       <c r="N48" t="str">
-        <v>TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="O48">
         <v>46</v>
@@ -3413,7 +3413,7 @@
         <v>0</v>
       </c>
       <c r="B49" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C49" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -3443,13 +3443,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L49" t="str">
-        <v>AGUILAR TORRES SARA VANESA</v>
+        <v/>
       </c>
       <c r="M49" t="str">
-        <v>SARA VANESA</v>
+        <v/>
       </c>
       <c r="N49" t="str">
-        <v>AGUILAR TORRES</v>
+        <v/>
       </c>
       <c r="O49">
         <v>21</v>
@@ -3469,7 +3469,7 @@
         <v>0</v>
       </c>
       <c r="B50" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C50" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -3499,13 +3499,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L50" t="str">
-        <v>BERNAL BECHARA LAILA CRISTINA</v>
+        <v/>
       </c>
       <c r="M50" t="str">
-        <v>LAILA CRISTINA</v>
+        <v/>
       </c>
       <c r="N50" t="str">
-        <v>BERNAL BECHARA</v>
+        <v/>
       </c>
       <c r="O50">
         <v>47</v>
@@ -3534,7 +3534,7 @@
         <v>0</v>
       </c>
       <c r="B51" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C51" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -3564,13 +3564,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L51" t="str">
-        <v>GUTIÉRREZ BARRERA EDUARD YEZID</v>
+        <v/>
       </c>
       <c r="M51" t="str">
-        <v>EDUARD YEZID</v>
+        <v/>
       </c>
       <c r="N51" t="str">
-        <v>GUTIÉRREZ BARRERA</v>
+        <v/>
       </c>
       <c r="O51">
         <v>52</v>
@@ -3599,7 +3599,7 @@
         <v>0</v>
       </c>
       <c r="B52" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C52" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -3629,13 +3629,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L52" t="str">
-        <v>SANCHEZ GARZON NATALI XIMENA</v>
+        <v/>
       </c>
       <c r="M52" t="str">
-        <v>NATALI XIMENA</v>
+        <v/>
       </c>
       <c r="N52" t="str">
-        <v>SANCHEZ GARZON</v>
+        <v/>
       </c>
       <c r="O52">
         <v>36</v>
@@ -3664,7 +3664,7 @@
         <v>0</v>
       </c>
       <c r="B53" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C53" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -3694,13 +3694,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L53" t="str">
-        <v>CORTES CORTES JAVIER EDUARDO</v>
+        <v/>
       </c>
       <c r="M53" t="str">
-        <v>JAVIER EDUARDO</v>
+        <v/>
       </c>
       <c r="N53" t="str">
-        <v>CORTES CORTES</v>
+        <v/>
       </c>
       <c r="O53">
         <v>55</v>
@@ -3729,7 +3729,7 @@
         <v>0</v>
       </c>
       <c r="B54" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C54" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -3759,13 +3759,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L54" t="str">
-        <v>TORRES SÁNCHEZ ERWIN GIOVANNI</v>
+        <v/>
       </c>
       <c r="M54" t="str">
-        <v>ERWIN GIOVANNI</v>
+        <v/>
       </c>
       <c r="N54" t="str">
-        <v>TORRES SÁNCHEZ</v>
+        <v/>
       </c>
       <c r="O54">
         <v>43</v>
@@ -3794,7 +3794,7 @@
         <v>0</v>
       </c>
       <c r="B55" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C55" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -3824,13 +3824,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L55" t="str">
-        <v>GARCIA GUZMAN NESTOR JAVIER</v>
+        <v/>
       </c>
       <c r="M55" t="str">
-        <v>NESTOR JAVIER</v>
+        <v/>
       </c>
       <c r="N55" t="str">
-        <v>GARCIA GUZMAN</v>
+        <v/>
       </c>
       <c r="O55">
         <v>35</v>
@@ -3859,7 +3859,7 @@
         <v>0</v>
       </c>
       <c r="B56" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C56" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -3889,13 +3889,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L56" t="str">
-        <v>PACHON MALDONADO DIEGO FERNANDO</v>
+        <v/>
       </c>
       <c r="M56" t="str">
-        <v>DIEGO FERNANDO</v>
+        <v/>
       </c>
       <c r="N56" t="str">
-        <v>PACHON MALDONADO</v>
+        <v/>
       </c>
       <c r="O56">
         <v>31</v>
@@ -3924,7 +3924,7 @@
         <v>0</v>
       </c>
       <c r="B57" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C57" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -3954,13 +3954,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L57" t="str">
-        <v>ACOSTA PEREZ NESTOR ENRIQUE</v>
+        <v/>
       </c>
       <c r="M57" t="str">
-        <v>NESTOR ENRIQUE</v>
+        <v/>
       </c>
       <c r="N57" t="str">
-        <v>ACOSTA PEREZ</v>
+        <v/>
       </c>
       <c r="O57">
         <v>37</v>
@@ -3989,7 +3989,7 @@
         <v>0</v>
       </c>
       <c r="B58" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C58" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -4019,13 +4019,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L58" t="str">
-        <v>CASTELLANOS TORRES JUAN DIEGO</v>
+        <v/>
       </c>
       <c r="M58" t="str">
-        <v>JUAN DIEGO</v>
+        <v/>
       </c>
       <c r="N58" t="str">
-        <v>CASTELLANOS TORRES</v>
+        <v/>
       </c>
       <c r="O58">
         <v>27</v>
@@ -4054,7 +4054,7 @@
         <v>0</v>
       </c>
       <c r="B59" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C59" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -4084,13 +4084,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L59" t="str">
-        <v>AHUMADA BELLO MARY LUZ</v>
+        <v/>
       </c>
       <c r="M59" t="str">
-        <v>MARY LUZ</v>
+        <v/>
       </c>
       <c r="N59" t="str">
-        <v>AHUMADA BELLO</v>
+        <v/>
       </c>
       <c r="O59">
         <v>46</v>
@@ -4119,7 +4119,7 @@
         <v>0</v>
       </c>
       <c r="B60" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C60" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -4149,13 +4149,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L60" t="str">
-        <v>GÓMEZ MURCIA JENNY JAZMIN</v>
+        <v/>
       </c>
       <c r="M60" t="str">
-        <v>JENNY JAZMIN</v>
+        <v/>
       </c>
       <c r="N60" t="str">
-        <v>GÓMEZ MURCIA</v>
+        <v/>
       </c>
       <c r="O60">
         <v>52</v>
@@ -4184,7 +4184,7 @@
         <v>0</v>
       </c>
       <c r="B61" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C61" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -4214,13 +4214,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L61" t="str">
-        <v>TORRES FORIGUA MONICA LORENA</v>
+        <v/>
       </c>
       <c r="M61" t="str">
-        <v>MONICA LORENA</v>
+        <v/>
       </c>
       <c r="N61" t="str">
-        <v>TORRES FORIGUA</v>
+        <v/>
       </c>
       <c r="O61">
         <v>37</v>
@@ -4249,7 +4249,7 @@
         <v>0</v>
       </c>
       <c r="B62" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C62" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -4279,13 +4279,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L62" t="str">
-        <v>VALIENTE TRIANA NANCY MILENA</v>
+        <v/>
       </c>
       <c r="M62" t="str">
-        <v>NANCY MILENA</v>
+        <v/>
       </c>
       <c r="N62" t="str">
-        <v>VALIENTE TRIANA</v>
+        <v/>
       </c>
       <c r="O62">
         <v>33</v>
@@ -4314,7 +4314,7 @@
         <v>0</v>
       </c>
       <c r="B63" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C63" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -4344,13 +4344,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L63" t="str">
-        <v>RODRIGUEZ PULGA SINDY LORENA</v>
+        <v/>
       </c>
       <c r="M63" t="str">
-        <v>SINDY LORENA</v>
+        <v/>
       </c>
       <c r="N63" t="str">
-        <v>RODRIGUEZ PULGA</v>
+        <v/>
       </c>
       <c r="O63">
         <v>41</v>
@@ -4379,7 +4379,7 @@
         <v>0</v>
       </c>
       <c r="B64" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C64" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -4409,13 +4409,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L64" t="str">
-        <v>RODRIGUEZ DIAZ JUAN DAVID</v>
+        <v/>
       </c>
       <c r="M64" t="str">
-        <v>JUAN DAVID</v>
+        <v/>
       </c>
       <c r="N64" t="str">
-        <v>RODRIGUEZ DIAZ</v>
+        <v/>
       </c>
       <c r="O64">
         <v>33</v>
@@ -4444,7 +4444,7 @@
         <v>0</v>
       </c>
       <c r="B65" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C65" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -4474,13 +4474,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L65" t="str">
-        <v>BOSA OCHOA CARLOS FELIPE</v>
+        <v/>
       </c>
       <c r="M65" t="str">
-        <v>CARLOS FELIPE</v>
+        <v/>
       </c>
       <c r="N65" t="str">
-        <v>BOSA OCHOA</v>
+        <v/>
       </c>
       <c r="O65">
         <v>55</v>
@@ -4509,7 +4509,7 @@
         <v>0</v>
       </c>
       <c r="B66" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C66" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -4539,13 +4539,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L66" t="str">
-        <v>GONZALEZ GONZALEZ ANDRES</v>
+        <v/>
       </c>
       <c r="M66" t="str">
-        <v>ANDRES</v>
+        <v/>
       </c>
       <c r="N66" t="str">
-        <v>GONZALEZ GONZALEZ</v>
+        <v/>
       </c>
       <c r="O66">
         <v>46</v>
@@ -4574,7 +4574,7 @@
         <v>0</v>
       </c>
       <c r="B67" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C67" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -4604,13 +4604,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L67" t="str">
-        <v>VERMAAS QUINTANA WILSON ERIC</v>
+        <v/>
       </c>
       <c r="M67" t="str">
-        <v>WILSON ERIC</v>
+        <v/>
       </c>
       <c r="N67" t="str">
-        <v>VERMAAS QUINTANA</v>
+        <v/>
       </c>
       <c r="O67">
         <v>37</v>
@@ -4639,7 +4639,7 @@
         <v>0</v>
       </c>
       <c r="B68" t="str">
-        <v>ADRIANA ASENCION TORRES ESPITIA</v>
+        <v/>
       </c>
       <c r="C68" t="str">
         <v>Experiencia Transformaciones que nos conectan Seccional Ubaté</v>
@@ -4669,13 +4669,13 @@
         <v>ACTIVA</v>
       </c>
       <c r="L68" t="str">
-        <v>LEÓN MURCIA GUILLERMO</v>
+        <v/>
       </c>
       <c r="M68" t="str">
-        <v>GUILLERMO</v>
+        <v/>
       </c>
       <c r="N68" t="str">
-        <v>LEÓN MURCIA</v>
+        <v/>
       </c>
       <c r="O68">
         <v>48</v>

</xml_diff>